<commit_message>
refactor: H4, build-cap names
</commit_message>
<xml_diff>
--- a/examples/unescap_training/inputs/scenarios/OSTRAM_Scenario_Inputs.xlsx
+++ b/examples/unescap_training/inputs/scenarios/OSTRAM_Scenario_Inputs.xlsx
@@ -6386,7 +6386,7 @@
     <t>BAU</t>
   </si>
   <si>
-    <t>add_max_cap_investment_lid_rule.py</t>
+    <t>build_cap_rule.py</t>
   </si>
   <si>
     <t>Base scenario</t>
@@ -6395,7 +6395,7 @@
     <t>A_Calibrated_BAU</t>
   </si>
   <si>
-    <t>set_retirement_schedule.py, add_max_cap_investment_lid_rule.py, set_min_capacity_floors.py, relax_interconnectors.py</t>
+    <t>set_retirement_schedule.py, build_cap_rule.py, set_min_capacity_floors.py, relax_interconnectors.py</t>
   </si>
   <si>
     <t>Test multi-script chain</t>
@@ -6404,7 +6404,7 @@
     <t>B_Optimised_VRE</t>
   </si>
   <si>
-    <t>set_retirement_schedule.py, add_max_cap_investment_lid_rule.py, relax_interconnectors.py, set_interconnector_direction.py, add_storage_min_investment.py</t>
+    <t>set_retirement_schedule.py, build_cap_rule.py, relax_interconnectors.py, set_interconnector_direction.py, add_storage_min_investment.py</t>
   </si>
   <si>
     <t>Loose VRE + open interconnectors (3x). No inheritance — independent solve from BAU base.</t>
@@ -6413,7 +6413,7 @@
     <t>C_Target_VRE</t>
   </si>
   <si>
-    <t>set_retirement_schedule.py, add_max_cap_investment_lid_rule.py, set_vre_targets.py, relax_interconnectors.py, add_storage_min_investment.py</t>
+    <t>set_retirement_schedule.py, build_cap_rule.py, set_vre_targets.py, relax_interconnectors.py, add_storage_min_investment.py</t>
   </si>
   <si>
     <t>NDC renewable targets. Independent solve from BAU base; hard dep is Executables/BAU_0/ProductionByTechnology.csv read by set_vre_targets.</t>

</xml_diff>